<commit_message>
feat: robustness - session with retires, .get() for API fields, CSV encoding
</commit_message>
<xml_diff>
--- a/RBCA_Register_2026-07-03.xlsx
+++ b/RBCA_Register_2026-07-03.xlsx
@@ -431,1080 +431,1080 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Registration Number</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>Company</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Registration Number</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>RBCP02281R2G</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>ACIVICO TRADED SERVICES LIMITED</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>RBCP02281R2G</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>RBCP01857Z0R</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>ACT BUILDING CONTROL LIMITED</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>RBCP01857Z0R</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>RBCP01972V4G</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>ADRIAN THOMAS BUILDING CONTROL LTD</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>RBCP01972V4G</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>RBCP01859B6C</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>ALIGN BUILDING CONTROL LTD</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>RBCP01859B6C</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>RBCP02331V3Y</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>ALL BUILDING CONTROL CERTIFICATION LIMITED</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>RBCP02331V3Y</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>RBCP01588F1G</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>Alpha Building Control Ltd</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>RBCP01588F1G</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>RBCP01489F0C</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>APPROVED BUILDING CONTROL LTD</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>RBCP01489F0C</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>RBCP01828S9Q</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>APPROVED INSPECTORS LIMITED</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>RBCP01828S9Q</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>RBCP03813W4W</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
           <t>ASK BUILDING CONTROL LTD</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>RBCP03813W4W</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>RBCP02306L1Y</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>ASSURE SURVEY LIMITED trading as ASSURE BUILDING CONTROL</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>RBCP02306L1Y</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>RBCP01855T3F</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
           <t>Ball &amp; Berry Ltd</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>RBCP01855T3F</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>RBCP06473Z4G</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
           <t>Blu Chip Compliance Ltd</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>RBCP06473Z4G</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>RBCP02269F0S</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
           <t>BLUEKEEP BUILDING CONTROL LIMITED</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>RBCP02269F0S</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>RBCP02307G5N</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
           <t>BUILD INSIGHT LTD</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>RBCP02307G5N</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>RBCP01845F5V</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
           <t>BUILDING CONSENTS LIMITED</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>RBCP01845F5V</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>RBCP06657X8R</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
           <t>Building Control Management Consultancy Limited</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>RBCP06657X8R</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>RBCP01664K2W</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
           <t>BUILDING CONTROL PARTNERSHIP LTD</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>RBCP01664K2W</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>RBCP01649X2X</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
           <t>BUILDING CONTROL SERVICES (APPROVED INSPECTORS) LIMITED</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>RBCP01649X2X</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>RBCP02227C5J</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
           <t>BUILDING CONTROL SURVEYORS LTD</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>RBCP02227C5J</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>RBCP01920C3H</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
           <t>Bureau Veritas Building Control UK Limited</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>RBCP01920C3H</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>RBCP01618S5D</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
           <t>C3 DESIGN APPROVALS LIMITED</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>RBCP01618S5D</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>RBCP02065Z6J</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
           <t>CLARKE BANKS (BUILDING CONTROL) LIMITED</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>RBCP02065Z6J</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>RBCP01766W4M</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
           <t>COAST 2 COAST BUILDING CONTROL LIMITED</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>RBCP01766W4M</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>RBCP01829C6Y</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
           <t>COMPLETE BUILDING CONTROL LTD</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>RBCP01829C6Y</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>RBCP01545D6F</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
           <t>COMPLIANCE BUILDING CONTROL LTD</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>RBCP01545D6F</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>RBCP06472W4G</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
           <t>Concept Construction Consultancy Ltd trading as Concept Building Control</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>RBCP06472W4G</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>RBCP01843P9H</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
           <t>CONFRERE BUILDING CONTROL LIMITED</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>RBCP01843P9H</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>RBCP01492Q6Z</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
           <t>COOK BROWN BUILDING CONTROL LTD</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>RBCP01492Q6Z</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>RBCP04290H0F</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
           <t>CORPORATE APPROVED INSPECTORS LTD</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>RBCP04290H0F</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>RBCP01648J1H</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
           <t>COUNTY BUILDING CONTROL LIMITED</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>RBCP01648J1H</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>RBCP05552L0S</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
           <t>DEEP BLUE BUILDING CONTROL CONSULTANCY LTD</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>RBCP05552L0S</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>RBCP01992C1D</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
           <t>DELTA CONSTRUCTION CONSULTANTS LTD</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>RBCP01992C1D</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>RBCP02268P9R</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
           <t>DUNWOODY BUILDING LEGISLATION LTD</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>RBCP02268P9R</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>RBCP04866Q6S</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
           <t>Ebor Mills Ltd</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>RBCP04866Q6S</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>RBCP02225M6S</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
           <t>EVOLVE BUILDING CONTROL CONSULTANTS LTD</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>RBCP02225M6S</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>RBCP01590X2P</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
           <t>GATEWAY BUILDING CONTROL LTD</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>RBCP01590X2P</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>RBCP06537M9K</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
           <t>Gatwick Building Control Ltd</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>RBCP06537M9K</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>RBCP02107H7N</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
           <t>H &amp; O Consulting Limited</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>RBCP02107H7N</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>RBCP02082M0C</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
           <t>HARWOOD BUILDING CONTROL LIMITED</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>RBCP02082M0C</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>RBCP02456G9W</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
           <t>ICW BUILDING CONTROL LTD</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>RBCP02456G9W</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>RBCP06532N0G</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
           <t>iM2 Building Approvers Ltd</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>RBCP06532N0G</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
+          <t>RBCP01586J8C</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
           <t>INTEGRAL BUILDING CONTROL SOLUTIONS LIMITED</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>RBCP01586J8C</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>RBCP01620W3H</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
           <t>JM PARTNERSHIP (SURVEYORS) LIMITED</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>RBCP01620W3H</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>RBCP05531V2X</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
           <t>JPI BUILDING CONTROL APPROVERS LTD</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>RBCP05531V2X</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
+          <t>RBCP06668K0W</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
           <t>K7 Building Compliance Ltd</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>RBCP06668K0W</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
+          <t>RBCP02119W9D</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
           <t>LHR BUILDING CONTROL SERVICES LIMITED</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>RBCP02119W9D</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
+          <t>RBCP02012Q0S</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
           <t>LONDON BUILDING CONTROL LIMITED</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>RBCP02012Q0S</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
+          <t>RBCP01557F1C</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
           <t>LSE BUILDING STANDARDS LTD</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>RBCP01557F1C</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
+          <t>RBCP01491C5C</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
           <t>MC Plan and Site Services Ltd</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>RBCP01491C5C</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
+          <t>RBCP01827C5W</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
           <t>MD WARRANTY SUPPORT SERVICES LIMITED trading as PREMIER GUARANTEE SURVEYORS</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>RBCP01827C5W</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
+          <t>RBCP01283W2M</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
           <t>MERIDIAN CONSULT LTD</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>RBCP01283W2M</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
+          <t>RBCP01947W1V</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
           <t>MFA BUILDING CONTROL LIMITED</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>RBCP01947W1V</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
+          <t>RBCP01962H0G</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
           <t>MIDLANDS BUILDING CONTROL CONSULTANCY LTD</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>RBCP01962H0G</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
+          <t>RBCP01723K2G</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
           <t>MORGAN WOLFF LIMITED</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>RBCP01723K2G</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
+          <t>RBCP03191K6S</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
           <t>MULLEE ASSOCIATES LIMITED</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>RBCP03191K6S</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
+          <t>RBCP01645Q4X</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
           <t>NHBC Building Control Services Limited</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>RBCP01645Q4X</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
+          <t>RBCP06525D2K</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
           <t>Nucleus Building Control Ltd</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>RBCP06525D2K</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
+          <t>RBCP02399T0D</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
           <t>ONSITE BUILDING CONTROL LTD</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>RBCP02399T0D</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
+          <t>RBCP06511V9F</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
           <t>Orbital Building Control Ltd</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>RBCP06511V9F</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
+          <t>RBCP01583G5L</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
           <t>OWL BUILDING CONTROL SOLUTIONS LIMITED</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>RBCP01583G5L</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
+          <t>RBCP01749S4Q</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
           <t>PRIME CONSTRUCTION CONSULTANTS LTD</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>RBCP01749S4Q</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
+          <t>RBCP02284F8Y</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
           <t>PRO BUILDING CONTROL LIMITED</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>RBCP02284F8Y</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
+          <t>RBCP02851W6V</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
           <t>PVM BUILDING CONTROL SERVICES LTD</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>RBCP02851W6V</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
+          <t>RBCP02575Q7D</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
           <t>QAI SERVICES LIMITED trading as QUADRANT BUILDING CONTROL</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>RBCP02575Q7D</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
+          <t>RBCP05860K2K</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
           <t>R360 Building Control Limited</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>RBCP05860K2K</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
+          <t>RBCP01585G4T</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
           <t>REGIONAL BUILDING CONTROL LIMITED trading as RBC LTD</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>RBCP01585G4T</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
+          <t>RBCP06216L3V</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
           <t>Restore Compliance Ltd</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>RBCP06216L3V</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
+          <t>RBCP02021D6S</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
           <t>RH BUILDING CONSULTANCY LIMITED</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>RBCP02021D6S</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
+          <t>RBCP02352V0K</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
           <t>RYAN PROPERTY CONSULTANTS LTD</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>RBCP02352V0K</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
+          <t>RBCP01529L0G</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
           <t>SALUS (BUILDING CONTROL AND FIRE SAFETY CONSULTANTS) LTD</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>RBCP01529L0G</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
+          <t>RBCP02570R4D</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
           <t>SHORE ENGINEERING LIMITED</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>RBCP02570R4D</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
+          <t>RBCP01753Z8Q</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
           <t>SOCOTEC Building Control Limited</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>RBCP01753Z8Q</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
+          <t>RBCP02682Y7Q</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
           <t>SPIRE BUILDING CONTROL SERVICES LIMITED</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>RBCP02682Y7Q</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
+          <t>RBCP01938F3N</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
           <t>STMC (BUILDING CONTROL) LTD</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>RBCP01938F3N</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
+          <t>RBCP01582M0N</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
           <t>Stroma Building Control Limited</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>RBCP01582M0N</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
+          <t>RBCP01544N5W</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
           <t>STUDIOUS LIMITED</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>RBCP01544N5W</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
+          <t>RBCP01748J9Z</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
           <t>SWECO BUILDING CONTROL LTD</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>RBCP01748J9Z</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
+          <t>RBCP05817B7T</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
           <t>SwellRock Construction Compliance Ltd</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>RBCP05817B7T</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
+          <t>RBCP01870K0X</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
           <t>TC BUILDING CONTROL LTD</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>RBCP01870K0X</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
+          <t>RBCP01663L8T</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
           <t>THAMES BUILDING CONTROL LIMITED</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>RBCP01663L8T</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
+          <t>RBCP01844K5Q</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
           <t>THE BUILDING INSPECTORS LIMITED</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>RBCP01844K5Q</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
+          <t>RBCP01823H9Z</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
           <t>TOP BUILDING CONTROL LTD</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>RBCP01823H9Z</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
+          <t>RBCP02457C8H</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
           <t>TOTAL BUILDING CONTROL LTD</t>
-        </is>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>RBCP02457C8H</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
+          <t>RBCP02009Y3H</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
           <t>TURTON BUILDING CONTROL LTD</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>RBCP02009Y3H</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
+          <t>RBCP05818C5P</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
           <t>Vanguard Building Compliance Ltd</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>RBCP05818C5P</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
+          <t>RBCP01502Q2N</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
           <t>VANTAGE BUILDING CONTROL LTD</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>RBCP01502Q2N</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
+          <t>RBCP02207N1J</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
           <t>WILKINSON CONSTRUCTION CONSULTANTS LTD</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>RBCP02207N1J</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
+          <t>RBCP02800N4V</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
           <t>YORKSHIRE BUILDING CONTROL LIMITED</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>RBCP02800N4V</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
+          <t>RBCP01759B9R</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
           <t>YORKSHIRE DALES BUILDING CONSULTANCY LTD trading as ENEVO BUILDING CONTROL</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>RBCP01759B9R</t>
         </is>
       </c>
     </row>

</xml_diff>